<commit_message>
end of day updates
</commit_message>
<xml_diff>
--- a/data/Bioenergetic parameters.xlsx
+++ b/data/Bioenergetic parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elizabethmchuron/Documents/GitHub/ak-nes-male/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elizabethmchuron/Documents/GitHub/NES-Male-AK/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0754D918-E993-4B46-9C62-0EAD9759CA29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09C799F6-5A60-5443-82C0-9096E3FBA95F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13960" yWindow="860" windowWidth="28040" windowHeight="17440" xr2:uid="{C553313F-25F1-4841-B1FE-82B0B5C15B3E}"/>
+    <workbookView xWindow="1380" yWindow="2180" windowWidth="19340" windowHeight="16060" xr2:uid="{C553313F-25F1-4841-B1FE-82B0B5C15B3E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="36">
   <si>
     <t>Parameter</t>
   </si>
@@ -110,9 +110,6 @@
     <t>Metabolizable energy</t>
   </si>
   <si>
-    <t>Value used by Jen</t>
-  </si>
-  <si>
     <t>popMult</t>
   </si>
   <si>
@@ -128,13 +125,25 @@
     <t>Chinn et al 2025</t>
   </si>
   <si>
-    <t>Crocker</t>
-  </si>
-  <si>
-    <t>Maresh et al</t>
-  </si>
-  <si>
     <t>Barbour 1993</t>
+  </si>
+  <si>
+    <t>FMRMult</t>
+  </si>
+  <si>
+    <t>Maresh et al 2014</t>
+  </si>
+  <si>
+    <t>Crocker unpubl</t>
+  </si>
+  <si>
+    <t>Value used in Maresh et al. 2014</t>
+  </si>
+  <si>
+    <t>MJ/kg0.75/day</t>
+  </si>
+  <si>
+    <t>Calculated from Table in Maresh et al 2014</t>
   </si>
 </sst>
 </file>
@@ -506,7 +515,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32233549-499E-5E46-A59B-B7C25E1B3614}">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
@@ -520,10 +529,10 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
         <v>27</v>
-      </c>
-      <c r="E1" t="s">
-        <v>28</v>
       </c>
       <c r="F1" t="s">
         <v>5</v>
@@ -540,10 +549,10 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>122.8</v>
+        <v>122.9</v>
       </c>
       <c r="C2">
-        <v>14.5</v>
+        <v>14.4</v>
       </c>
       <c r="D2">
         <v>102</v>
@@ -558,7 +567,7 @@
         <v>18</v>
       </c>
       <c r="H2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
@@ -566,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>1256</v>
+        <v>1291</v>
       </c>
       <c r="C3">
         <v>276</v>
@@ -575,7 +584,7 @@
         <v>752</v>
       </c>
       <c r="E3">
-        <v>1860</v>
+        <v>1861</v>
       </c>
       <c r="F3" t="s">
         <v>7</v>
@@ -584,7 +593,7 @@
         <v>19</v>
       </c>
       <c r="H3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -592,7 +601,7 @@
         <v>8</v>
       </c>
       <c r="B4">
-        <v>70</v>
+        <v>69.8</v>
       </c>
       <c r="C4">
         <v>23.2</v>
@@ -610,12 +619,12 @@
         <v>20</v>
       </c>
       <c r="H4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B5">
         <v>1.3</v>
@@ -641,59 +650,68 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B6">
-        <v>0.11600000000000001</v>
+        <v>0.39</v>
+      </c>
+      <c r="C6">
+        <v>0.1</v>
       </c>
       <c r="D6">
-        <v>6.4000000000000001E-2</v>
+        <v>0.27</v>
       </c>
       <c r="E6">
-        <v>0.17699999999999999</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="F6" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="G6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B7">
-        <v>0.83</v>
+        <v>0.11600000000000001</v>
+      </c>
+      <c r="D7">
+        <v>6.4000000000000001E-2</v>
+      </c>
+      <c r="E7">
+        <v>0.17699999999999999</v>
       </c>
       <c r="F7" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H7" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="B8">
-        <v>194903</v>
-      </c>
-      <c r="D8">
-        <v>170185</v>
-      </c>
-      <c r="E8">
-        <v>233677</v>
+        <v>0.83</v>
+      </c>
+      <c r="F8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" t="s">
+        <v>23</v>
       </c>
       <c r="H8" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -701,10 +719,27 @@
         <v>25</v>
       </c>
       <c r="B9">
+        <v>194903</v>
+      </c>
+      <c r="D9">
+        <v>170185</v>
+      </c>
+      <c r="E9">
+        <v>233677</v>
+      </c>
+      <c r="H9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10">
         <v>3.7699999999999997E-2</v>
       </c>
-      <c r="H9" t="s">
-        <v>29</v>
+      <c r="H10" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>